<commit_message>
admin placement complate with export excel
</commit_message>
<xml_diff>
--- a/backend/enquiries.xlsx
+++ b/backend/enquiries.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -455,9 +455,121 @@
         <v>Undergraduate</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>frdyrty</v>
+      </c>
+      <c r="C5" t="str">
+        <v>6578765876</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Diploma</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>hkuio,l</v>
+      </c>
+      <c r="C6" t="str">
+        <v>5745687689</v>
+      </c>
+      <c r="D6" t="str">
+        <v>12th</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>mjghj</v>
+      </c>
+      <c r="C7" t="str">
+        <v>6754444444</v>
+      </c>
+      <c r="D7" t="str">
+        <v>12th</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>yhjiyg</v>
+      </c>
+      <c r="C8" t="str">
+        <v>765984633</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Diploma</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>jmlllllh</v>
+      </c>
+      <c r="C9" t="str">
+        <v>76896846</v>
+      </c>
+      <c r="D9" t="str">
+        <v>12th</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>hgjg</v>
+      </c>
+      <c r="C10" t="str">
+        <v>678888888</v>
+      </c>
+      <c r="D10" t="str">
+        <v>12th</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>gfdj</v>
+      </c>
+      <c r="C11" t="str">
+        <v>6784567478</v>
+      </c>
+      <c r="D11" t="str">
+        <v>12th</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>jhk</v>
+      </c>
+      <c r="C12" t="str">
+        <v>687574356</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Diploma</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>